<commit_message>
update cache file, SetDataSource
</commit_message>
<xml_diff>
--- a/ProductTest.Presentation/Template/Product/ProductTemplate.xlsx
+++ b/ProductTest.Presentation/Template/Product/ProductTemplate.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>STT</t>
   </si>
@@ -69,6 +69,48 @@
   </si>
   <si>
     <t>HẾT HẠN</t>
+  </si>
+  <si>
+    <t>&amp;=&amp;=Row()-1</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].ID</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].CODE</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].NAME</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].DESCRIPTION</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].CATEGORY</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].PRICE</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].TAXRATE</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].STOCK</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].SUPPLERID</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].ISACTIVE</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].CREATEDAT</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].UPDATEDAT</t>
+  </si>
+  <si>
+    <t>&amp;=[Product].EXPIREDDT</t>
   </si>
 </sst>
 </file>
@@ -717,15 +759,18 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1263,101 +1308,146 @@
   <dimension ref="A1:N16"/>
   <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" customWidth="1"/>
-    <col min="2" max="2" width="19.4285714285714" customWidth="1"/>
-    <col min="3" max="3" width="23.8571428571429" customWidth="1"/>
-    <col min="4" max="4" width="25.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="12.8571428571429" customWidth="1"/>
-    <col min="6" max="6" width="19.8571428571429" customWidth="1"/>
-    <col min="7" max="7" width="10.5714285714286" customWidth="1"/>
-    <col min="8" max="8" width="18.5714285714286" customWidth="1"/>
-    <col min="9" max="9" width="14.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
-    <col min="11" max="11" width="19.2857142857143" customWidth="1"/>
-    <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="13" max="13" width="26.2857142857143" customWidth="1"/>
-    <col min="14" max="14" width="15.1428571428571" customWidth="1"/>
+    <col min="1" max="1" width="34.6190476190476" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.4285714285714" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.8571428571429" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.7142857142857" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31" style="1" customWidth="1"/>
+    <col min="6" max="6" width="32.1428571428571" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.1428571428571" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.4285714285714" style="1" customWidth="1"/>
+    <col min="9" max="9" width="33.4285714285714" style="1" customWidth="1"/>
+    <col min="10" max="10" width="24" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.2857142857143" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23" style="1" customWidth="1"/>
+    <col min="13" max="13" width="26.2857142857143" style="1" customWidth="1"/>
+    <col min="14" max="14" width="25.4952380952381" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.2857142857143" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.5" spans="1:14">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="24" customHeight="1" spans="1:14">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="2" ht="27" customHeight="1" spans="1:14">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="16.5" spans="1:14">
-      <c r="C5" s="2"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" ht="16.5" spans="1:14">
-      <c r="C6" s="2"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" ht="16.5" spans="1:14">
-      <c r="C7" s="2"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" ht="16.5" spans="1:14">
-      <c r="C8" s="2"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" ht="16.5" spans="1:14">
-      <c r="C9" s="2"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" ht="16.5" spans="1:14">
-      <c r="C10" s="2"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" ht="16.5" spans="1:14">
-      <c r="C11" s="2"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" ht="16.5" spans="1:14">
-      <c r="C12" s="2"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="13" ht="16.5" spans="1:14">
-      <c r="C13" s="2"/>
+      <c r="C13" s="3"/>
     </row>
     <row r="14" ht="16.5" spans="1:14">
-      <c r="C14" s="2"/>
+      <c r="C14" s="3"/>
     </row>
     <row r="15" ht="16.5" spans="1:14">
-      <c r="C15" s="2"/>
+      <c r="C15" s="3"/>
     </row>
     <row r="16" ht="16.5" spans="1:14">
-      <c r="C16" s="2"/>
+      <c r="C16" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>